<commit_message>
data: add PVcomBank bank mapping
</commit_message>
<xml_diff>
--- a/phieu-ck-data.xlsx
+++ b/phieu-ck-data.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9.5546875" customWidth="1" min="1" max="1"/>
@@ -1897,6 +1897,38 @@
       <c r="F48" t="inlineStr">
         <is>
           <t>TIMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>79360001-</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>970412</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Ngân hàng TMCP Đại Chúng Việt Nam (PVcomBank) - PVC</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Ngân hàng TMCP Đại Chúng Việt Nam</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>PVcomBank</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>PVC</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2148,6 @@
           <t>970422</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2376,7 +2407,6 @@
           <t>546034</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2394,7 +2424,6 @@
           <t>546035</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2412,7 +2441,6 @@
           <t>971011</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2430,7 +2458,6 @@
           <t>971005</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2448,7 +2475,6 @@
           <t>963388</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2466,7 +2492,6 @@
           <t>963369</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2484,7 +2509,6 @@
           <t>963368</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2502,7 +2526,6 @@
           <t>963311</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2542,7 +2565,6 @@
           <t>977777</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2560,7 +2582,6 @@
           <t>971100</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2600,7 +2621,6 @@
           <t>963326</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2618,7 +2638,6 @@
           <t>971032</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2636,7 +2655,6 @@
           <t>971034</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2654,7 +2672,6 @@
           <t>971101</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2664,7 +2681,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Đại chúng Việt Nam (PVC)</t>
+          <t>Đại chúng Việt Nam (PVcomBank/PVC)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2887,7 +2904,6 @@
           <t>Phát triển Việt Nam (VDB)</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
           <t>01208001</t>
@@ -3086,7 +3102,6 @@
           <t>963399</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3104,7 +3119,6 @@
           <t>971133</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3205,7 +3219,6 @@
           <t>Malayan Banking Berhad (MALAYAN)</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
           <t>79635001</t>
@@ -3223,7 +3236,6 @@
           <t>BPCE IOM (NATIXIS)</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
           <t>79601001</t>
@@ -3263,7 +3275,6 @@
           <t>NH MUFG BANK LTD CN HA NOI</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
           <t>01653001</t>
@@ -3391,7 +3402,6 @@
           <t>MIZUHO BANK HA NOI (MIZUHO)</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
           <t>01613001</t>
@@ -3519,7 +3529,6 @@
           <t>TNHH MTV ANZ Việt Nam (ANZ)</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
           <t>01602002</t>
@@ -3537,7 +3546,6 @@
           <t>Bangkok Đại chúng TNHH (BANGKOK)</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
           <t>01667001</t>
@@ -3599,7 +3607,6 @@
           <t>Xây dựng Trung Quốc (CCB)</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr">
         <is>
           <t>79611001</t>
@@ -3617,7 +3624,6 @@
           <t>TNHH CTBC (CHINATRUST)</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
           <t>79629001</t>
@@ -3833,7 +3839,6 @@
           <t>May Bank (MAYBANK)</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
           <t>01609001</t>
@@ -3851,7 +3856,6 @@
           <t>MEGA ICBC (MEGA)</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
           <t>79623001</t>
@@ -3869,7 +3873,6 @@
           <t>The Shanghai Commercial &amp; Savings (SHANGHAI)</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr">
         <is>
           <t>75606001</t>
@@ -3887,7 +3890,6 @@
           <t>OVERSEA - CHINESE BANKING CORP (CHINESE)</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
           <t>79625001</t>
@@ -3905,7 +3907,6 @@
           <t>SUMITOMO MITSUI BANKING CORPORATION (SMBC)</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
           <t>01636001</t>
@@ -3923,7 +3924,6 @@
           <t>Taipei Fubon (TAIPEI)</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
           <t>01642001</t>
@@ -4007,7 +4007,6 @@
           <t>Citibank TP.Hồ Chí Minh (CITIBANK)</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr">
         <is>
           <t>79654001</t>
@@ -4025,7 +4024,6 @@
           <t>MIZUHO BANK TP HO CHI MINH (MIZUHO)</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr"/>
       <c r="D95" t="inlineStr">
         <is>
           <t>79639001</t>
@@ -4043,7 +4041,6 @@
           <t>NH AGRICULTURAL BANK OF CHINA LTD HN</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
           <t>01664001</t>
@@ -4083,7 +4080,6 @@
           <t>FIRST COMMERCIAL BANK CN TP HCM</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
           <t>79630001</t>
@@ -4101,7 +4097,6 @@
           <t>NH MUFG BANK LTD CN TP HCM</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
           <t>79622001</t>
@@ -4163,7 +4158,6 @@
           <t>BANK OF COMMUNICATIONS (COMMUNICATION)</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
           <t>79615001</t>
@@ -4203,7 +4197,6 @@
           <t>COMMONWEALTH BANK (COMMONWEALTH)</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
           <t>79643001</t>
@@ -4221,7 +4214,6 @@
           <t>FIRST COMMERCIAL BANK CN HA NOI</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
           <t>01608001</t>
@@ -4239,7 +4231,6 @@
           <t>HUA NAN COMMERCIAL BANK (HUA NAN)</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr"/>
       <c r="D106" t="inlineStr">
         <is>
           <t>79640001</t>
@@ -4257,7 +4248,6 @@
           <t>JPMORGAN CHASE (MCB)</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
           <t>79627001</t>
@@ -4280,7 +4270,6 @@
           <t>971025</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: update full bank list from VietQR review
</commit_message>
<xml_diff>
--- a/phieu-ck-data.xlsx
+++ b/phieu-ck-data.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9.5546875" customWidth="1" min="1" max="1"/>
@@ -496,8 +496,10 @@
           <t>01203001-</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>970436</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>970436</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -526,8 +528,10 @@
           <t>01309001-</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>970432</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>970432</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -556,8 +560,10 @@
           <t>01310001-</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>970407</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>970407</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -586,8 +592,10 @@
           <t>01202001-</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>970418</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>970418</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -616,8 +624,10 @@
           <t>01311003-</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>970422</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>970422</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -646,8 +656,10 @@
           <t>01201001-</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>970415</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>970415</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -676,8 +688,10 @@
           <t>01204001-</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>970405</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>970405</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -706,8 +720,10 @@
           <t>01307001-</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>970416</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>970416</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -736,8 +752,10 @@
           <t>01348002-</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>970443</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>970443</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -766,8 +784,10 @@
           <t>79321001-</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>970437</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>970437</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -796,8 +816,10 @@
           <t>01357001-</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>970449</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>970449</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -826,8 +848,10 @@
           <t>79314013-</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>970441</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>970441</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -856,8 +880,10 @@
           <t>01317001-</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>970440</v>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>970440</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -886,8 +912,10 @@
           <t>79358001-</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>970423</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>970423</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -916,8 +944,10 @@
           <t>01302001-</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>970426</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>970426</t>
+        </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -946,8 +976,10 @@
           <t>01207001-</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>999888</v>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>999888</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -976,8 +1008,10 @@
           <t>79333001-</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>970448</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>970448</t>
+        </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1006,8 +1040,10 @@
           <t>79303001-</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>970403</v>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>970403</t>
+        </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1036,8 +1072,10 @@
           <t>79305001-</t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>970431</v>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>970431</t>
+        </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1066,8 +1104,10 @@
           <t>79334001-</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>970429</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>970429</t>
+        </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1096,8 +1136,10 @@
           <t>79306001-</t>
         </is>
       </c>
-      <c r="B22" t="n">
-        <v>970428</v>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>970428</t>
+        </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1126,8 +1168,10 @@
           <t>01663001-</t>
         </is>
       </c>
-      <c r="B23" t="n">
-        <v>970457</v>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>970457</t>
+        </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1156,8 +1200,10 @@
           <t>01352002-</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>970419</v>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>970419</t>
+        </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1186,8 +1232,10 @@
           <t>01323002-</t>
         </is>
       </c>
-      <c r="B25" t="n">
-        <v>970425</v>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>970425</t>
+        </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1216,8 +1264,10 @@
           <t>79665001-</t>
         </is>
       </c>
-      <c r="B26" t="n">
-        <v>970458</v>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>970458</t>
+        </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1246,8 +1296,10 @@
           <t>01313007-</t>
         </is>
       </c>
-      <c r="B27" t="n">
-        <v>970409</v>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>970409</t>
+        </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1276,8 +1328,10 @@
           <t>01617001-</t>
         </is>
       </c>
-      <c r="B28" t="n">
-        <v>458761</v>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>458761</t>
+        </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1306,8 +1360,10 @@
           <t>79356001-</t>
         </is>
       </c>
-      <c r="B29" t="n">
-        <v>970433</v>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>970433</t>
+        </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1336,8 +1392,10 @@
           <t>01604001-</t>
         </is>
       </c>
-      <c r="B30" t="n">
-        <v>970410</v>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>970410</t>
+        </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1366,8 +1424,10 @@
           <t>79616001-</t>
         </is>
       </c>
-      <c r="B31" t="n">
-        <v>970424</v>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>970424</t>
+        </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1396,8 +1456,10 @@
           <t>01355002-</t>
         </is>
       </c>
-      <c r="B32" t="n">
-        <v>970427</v>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>970427</t>
+        </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1426,8 +1488,10 @@
           <t>01341001-</t>
         </is>
       </c>
-      <c r="B33" t="n">
-        <v>970430</v>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>970430</t>
+        </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1456,8 +1520,10 @@
           <t>01661001-</t>
         </is>
       </c>
-      <c r="B34" t="n">
-        <v>422589</v>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>422589</t>
+        </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1486,8 +1552,10 @@
           <t>91353001-</t>
         </is>
       </c>
-      <c r="B35" t="n">
-        <v>970452</v>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>970452</t>
+        </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1516,8 +1584,10 @@
           <t>79308001-</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>970400</v>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>970400</t>
+        </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1546,8 +1616,10 @@
           <t>01502001-</t>
         </is>
       </c>
-      <c r="B37" t="n">
-        <v>970434</v>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>970434</t>
+        </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1576,8 +1648,10 @@
           <t>01359001-</t>
         </is>
       </c>
-      <c r="B38" t="n">
-        <v>970438</v>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>970438</t>
+        </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1606,8 +1680,10 @@
           <t>01505001-</t>
         </is>
       </c>
-      <c r="B39" t="n">
-        <v>970421</v>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>970421</t>
+        </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1636,8 +1712,10 @@
           <t>01901001-</t>
         </is>
       </c>
-      <c r="B40" t="n">
-        <v>970446</v>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>970446</t>
+        </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1666,8 +1744,10 @@
           <t>79603001-</t>
         </is>
       </c>
-      <c r="B41" t="n">
-        <v>970442</v>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>970442</t>
+        </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1696,8 +1776,10 @@
           <t>79304001-</t>
         </is>
       </c>
-      <c r="B42" t="n">
-        <v>970406</v>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>970406</t>
+        </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1726,8 +1808,10 @@
           <t>01319001-</t>
         </is>
       </c>
-      <c r="B43" t="n">
-        <v>970414</v>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>970414</t>
+        </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1756,8 +1840,10 @@
           <t>01320001-</t>
         </is>
       </c>
-      <c r="B44" t="n">
-        <v>970408</v>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>970408</t>
+        </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1786,8 +1872,10 @@
           <t>01016001-</t>
         </is>
       </c>
-      <c r="B45" t="n">
-        <v>971005</v>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>971005</t>
+        </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1816,8 +1904,10 @@
           <t>80339001-</t>
         </is>
       </c>
-      <c r="B46" t="n">
-        <v>970444</v>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>970444</t>
+        </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1846,8 +1936,10 @@
           <t>01010001-</t>
         </is>
       </c>
-      <c r="B47" t="n">
-        <v>546034</v>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>546034</t>
+        </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1876,8 +1968,10 @@
           <t>01012001-</t>
         </is>
       </c>
-      <c r="B48" t="n">
-        <v>963388</v>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>963388</t>
+        </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1929,6 +2023,530 @@
       <c r="F49" t="inlineStr">
         <is>
           <t>PVC</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>79327001-</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>970454</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Ngân hàng TMCP Bản Việt (VietCapitalBank) - VCCB</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Ngân hàng TMCP Bản Việt</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>VietCapitalBank</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>VCCB</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>01011001-</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>546035</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>TMCP Việt Nam Thịnh Vượng - Ngân hàng số Ubank by VPBank (Ubank) - Ubank</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>TMCP Việt Nam Thịnh Vượng - Ngân hàng số Ubank by VPBank</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Ubank</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Ubank</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>971011</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>VNPT Money (VNPTMoney) - VNPTMONEY</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>VNPT Money</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>VNPTMoney</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>VNPTMONEY</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>971025</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>CTCP Dịch Vụ Di Động Trực Tuyến (MoMo) - momo</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>CTCP Dịch Vụ Di Động Trực Tuyến</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>MoMo</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>momo</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>971133</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Ngân hàng TMCP Đại Chúng Việt Nam Ngân hàng số (PVcomBank Pay) - PVDB</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Ngân hàng TMCP Đại Chúng Việt Nam Ngân hàng số</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>PVcomBank Pay</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>PVDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>79669001-</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>668888</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Ngân hàng Đại chúng TNHH Kasikornbank (KBank) - KBank</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Ngân hàng Đại chúng TNHH Kasikornbank</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>KBank</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>KBank</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>01017001-</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>977777</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Công ty Tài chính TNHH MTV Mirae Asset (Việt Nam)  (MAFC) - MAFC</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Công ty Tài chính TNHH MTV Mirae Asset (Việt Nam)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>MAFC</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>MAFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>01626001-</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>970467</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Ngân hàng KEB Hana – Chi nhánh Hà Nội (KEBHANAHN) - KEBHANAHN</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Ngân hàng KEB Hana – Chi nhánh Hà Nội</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>KEBHANAHN</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>KEBHANAHN</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>79656001-</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>970466</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Ngân hàng KEB Hana – Chi nhánh Thành phố Hồ Chí Minh (KEBHanaHCM) - KEBHANAHCM</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Ngân hàng KEB Hana – Chi nhánh Thành phố Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>KEBHanaHCM</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>KEBHANAHCM</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>01605001-</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>533948</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Ngân hàng Citibank, N.A. - Chi nhánh Hà Nội (Citibank) - CITIBANK</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Ngân hàng Citibank, N.A. - Chi nhánh Hà Nội</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Citibank</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>CITIBANK</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>79650001-</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>796500</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>DBS Bank Ltd - Chi nhánh Thành phố Hồ Chí Minh (DBSBank) - DBS</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>DBS Bank Ltd - Chi nhánh Thành phố Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>DBSBank</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>DBS</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>79631001-</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>970463</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Ngân hàng Kookmin - Chi nhánh Thành phố Hồ Chí Minh (KookminHCM) - KBHCM</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Ngân hàng Kookmin - Chi nhánh Thành phố Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>KookminHCM</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>KBHCM</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>01666001-</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>970462</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Ngân hàng Kookmin - Chi nhánh Hà Nội (KookminHN) - KBHN</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Ngân hàng Kookmin - Chi nhánh Hà Nội</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>KookminHN</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>KBHN</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>01652001-</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>970455</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Ngân hàng Công nghiệp Hàn Quốc - Chi nhánh Hà Nội (IBKHN) - IBK - HN</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Ngân hàng Công nghiệp Hàn Quốc - Chi nhánh Hà Nội</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>IBKHN</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>IBK - HN</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>970456</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Ngân hàng Công nghiệp Hàn Quốc - Chi nhánh TP. Hồ Chí Minh (IBKHCM) - IBK - HCM</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Ngân hàng Công nghiệp Hàn Quốc - Chi nhánh TP. Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>IBKHCM</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>IBK - HCM</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>01662001-</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>801011</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Ngân hàng Nonghyup - Chi nhánh Hà Nội (Nonghyup) - NHB HN</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Ngân hàng Nonghyup - Chi nhánh Hà Nội</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Nonghyup</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>NHB HN</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>970439</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Ngân hàng TNHH MTV Public Việt Nam (PublicBank) - PBVN</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Ngân hàng TNHH MTV Public Việt Nam</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>PublicBank</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>PBVN</t>
         </is>
       </c>
     </row>

</xml_diff>